<commit_message>
Run Tripadvisor scrape for pages 2-4
Co-authored-by: 吴志中 <wuzhizhong1@xdf.cn>
</commit_message>
<xml_diff>
--- a/attractionsFromPage.xlsx
+++ b/attractionsFromPage.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B150"/>
+  <dimension ref="A1:B91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,1491 +430,901 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>151</v>
+        <v>31</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>中央大街步行街</t>
+          <t>上窰民俗文物馆</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>152</v>
+        <v>32</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>印象丽江</t>
+          <t>国际眼镜城</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>153</v>
+        <v>33</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>崇圣寺三塔</t>
+          <t>西藏高原旅游的一日游</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>154</v>
+        <v>34</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>文殊院</t>
+          <t>香港旅游发展局</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>155</v>
+        <v>35</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>香港西贡</t>
+          <t>Sandbox - 沙盒 VR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>156</v>
+        <v>36</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>广州地铁</t>
+          <t>张家界国家森林公园</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>157</v>
+        <v>37</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>上海城市历史发展陈列馆</t>
+          <t>布达拉宫</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>158</v>
+        <v>38</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>杭州宋城</t>
+          <t>L&amp;K裁缝</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>159</v>
+        <v>39</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Beijing Airport Layover Tour</t>
+          <t>南外滩轻纺面料市场</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>鹿回头公园</t>
+          <t>黄花城长城</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>161</v>
+        <v>41</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>狮子林</t>
+          <t>Xianggong Mountain</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>162</v>
+        <v>42</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>陈家祠</t>
+          <t>云冈石窟</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>163</v>
+        <v>43</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>网师园</t>
+          <t>大熊猫保护研究中心都江堰基地</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>164</v>
+        <v>44</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>中国丽江古城</t>
+          <t>九寨沟自然保护区</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>165</v>
+        <v>45</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>798艺术区</t>
+          <t>黑暗中对话</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>166</v>
+        <v>46</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>香港海事博物馆</t>
+          <t>南莲园池</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>167</v>
+        <v>47</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>东方明珠</t>
+          <t>箭扣长城</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>168</v>
+        <v>48</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>崂山自然风景区</t>
+          <t>亚特兰蒂斯水世界</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>169</v>
+        <v>49</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>汉阳陵</t>
+          <t>黄山</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>170</v>
+        <v>50</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>峨眉山</t>
+          <t>龙脊梯田</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>171</v>
+        <v>51</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>同里古镇</t>
+          <t>张家界天门山</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>172</v>
+        <v>52</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>豫园</t>
+          <t>龙门石窟</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>173</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>大馆</t>
+          <t>哈尔滨冰雪大世界</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>174</v>
+        <v>54</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>云南石林地质公园</t>
+          <t>居庸关长城</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>175</v>
+        <v>55</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>天一阁</t>
+          <t>司马台长城</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>176</v>
+        <v>56</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>西湖花港观鱼公园</t>
+          <t>泸沽湖</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>177</v>
+        <v>57</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>金茂大厦</t>
+          <t>张家界武陵源风景名胜区</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>178</v>
+        <v>58</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>回坊风情街</t>
+          <t>龙脊</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>179</v>
+        <v>59</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>花城广场</t>
+          <t>外滩万国建筑博览</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>颐和园佛香阁</t>
+          <t>志莲净苑</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>181</v>
+        <v>61</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>平江路</t>
+          <t>悬空寺</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>182</v>
+        <v>62</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>虎丘</t>
+          <t>Art Alba Gallery</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>183</v>
+        <v>63</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>青海湖</t>
+          <t>Real China Travel</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>184</v>
+        <v>64</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>香港文化博物馆</t>
+          <t>莫高窟</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>185</v>
+        <v>65</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>太阳岛</t>
+          <t>拉萨大昭寺</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>186</v>
+        <v>66</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>鸣沙山</t>
+          <t>成都地铁</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>187</v>
+        <v>67</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>玉佛禅寺</t>
+          <t>跑马地赛马场</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>188</v>
+        <v>68</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>凤凰古城</t>
+          <t>慈山寺</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>189</v>
+        <v>69</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>昆明龙门</t>
+          <t>遇龙河</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>190</v>
+        <v>70</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>金沙遗址博物馆</t>
+          <t>上海中心大厦</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>191</v>
+        <v>71</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>中华恐龙园</t>
+          <t>长隆国际马戏大剧院</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>192</v>
+        <v>72</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>明孝陵</t>
+          <t>上海犹太难民纪念馆</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>193</v>
+        <v>73</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>郑家大屋</t>
+          <t>张掖丹霞地质文化公园</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>194</v>
+        <v>74</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>旧城</t>
+          <t>雍和宫</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>195</v>
+        <v>75</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Happy Dragon Tour</t>
+          <t>北京八达岭长城</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>196</v>
+        <v>76</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>南京城墙(明城墙)</t>
+          <t>香港电车（叮叮车）</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>197</v>
+        <v>77</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>珠海长隆海洋王国</t>
+          <t>景山公园</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>新濠天地</t>
+          <t>漓江景区</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>周庄水乡</t>
+          <t>哲蚌寺</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alex's Epic Xian的一日游</t>
+          <t>西湖</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>201</v>
+        <v>81</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>澳门历史城区</t>
+          <t>飞来峰</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>202</v>
+        <v>82</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>留园</t>
+          <t>国家大剧院</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>203</v>
+        <v>83</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>香港历史博物馆</t>
+          <t>u-bestour</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>204</v>
+        <v>84</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>陕西历史博物馆</t>
+          <t>湖北省博物馆</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>205</v>
+        <v>85</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>苏州博物馆</t>
+          <t>华山</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>206</v>
+        <v>86</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>八大关</t>
+          <t>磁悬浮列车</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>207</v>
+        <v>87</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>午门</t>
+          <t>太和殿</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>208</v>
+        <v>88</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>珠穆朗玛峰基地营</t>
+          <t>长隆野生动物园</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>209</v>
+        <v>89</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>两江四湖景区</t>
+          <t>上海宣传画艺术中心</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>211</v>
+        <v>90</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>长洲岛</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>212</v>
+        <v>91</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>白云山</t>
+          <t>南山寺</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>213</v>
+        <v>92</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>峨眉山金顶</t>
+          <t>香港维多利亚海港</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>214</v>
+        <v>93</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>澳门大熊猫馆</t>
+          <t>北海公园</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>215</v>
+        <v>94</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>朱家角古镇</t>
+          <t>Mary’s Xian Tours</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>216</v>
+        <v>95</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>扎什伦布寺</t>
+          <t>云台山地质公园</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>217</v>
+        <v>96</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>古北水镇</t>
+          <t>猫之茶房</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>218</v>
+        <v>97</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>武汉东湖</t>
+          <t>八角街</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>219</v>
+        <v>98</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>大雁塔</t>
+          <t>祈年殿</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>220</v>
+        <v>99</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>锦绣中华·民俗村</t>
+          <t>云南沙溪古镇</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>221</v>
+        <v>100</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>大雁塔北广场</t>
+          <t>大屿山</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>222</v>
+        <v>101</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>青岛啤酒博物馆</t>
+          <t>深圳莲花山公园</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>223</v>
+        <v>102</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>西塘古镇</t>
+          <t>虎跳峡</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>224</v>
+        <v>103</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>沙面岛</t>
+          <t>西安城墙</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>225</v>
+        <v>104</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>黄龙名胜风景区</t>
+          <t>滨江大道</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>226</v>
+        <v>105</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>尖沙咀海滨长廊</t>
+          <t>天际100香港观景台</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>227</v>
+        <v>106</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>星海广场</t>
+          <t>观光缆车</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>228</v>
+        <v>107</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>故宫九龙壁</t>
+          <t>上海环球金融中心</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>229</v>
+        <v>108</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Guangzhou Private Local Tour Guide-Lorena</t>
+          <t>浦东新区</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>230</v>
+        <v>109</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>上海人文历史地貌区</t>
+          <t>成都大熊猫繁育研究基地</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>231</v>
+        <v>110</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>复兴公园</t>
+          <t>朝阳剧场</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>232</v>
+        <v>111</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>岳麓山</t>
+          <t>平遥古城</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>233</v>
+        <v>112</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>大澳</t>
+          <t>香港公园</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>234</v>
+        <v>113</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>外滩城市雕塑群</t>
+          <t>苏州古典园林</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>235</v>
+        <v>114</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>广州图书馆</t>
+          <t>万佛寺</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>236</v>
+        <v>115</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>大芬油画村</t>
+          <t>龙华寺</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>237</v>
+        <v>116</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>趵突泉公园</t>
+          <t>上海自然博物馆(静安新馆)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>238</v>
+        <v>117</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>南丫岛</t>
+          <t>长隆欢乐世界</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>239</v>
+        <v>118</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>南普陀寺</t>
+          <t>宝莲禅寺</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>240</v>
+        <v>119</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>金鸡湖</t>
+          <t>狮子亭观景台</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>241</v>
+        <v>120</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>九龙公园</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>242</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Travel Beijing Guide</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>243</v>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>三清山</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>244</v>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>SoHo 荷南美食区</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>245</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>后海</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>246</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>普陀山</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>247</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>COCO PARK</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>248</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>西安博物院</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>249</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>冈仁波齐峰</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>250</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>赤柱</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>251</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Beijing Impression Tours</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>252</v>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>厦门大学</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>253</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>孔庙和国子监博物馆</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>254</v>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>成都人民公园</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>255</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>束河古镇</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>256</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>China Educational Tours</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>257</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>石室圣心大教堂</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>258</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>杜甫草堂</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>259</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>圆明园</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>260</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>祖庙</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>261</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>珠江</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>262</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>上海虹桥火车站</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>263</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>元阳梯田</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>264</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>鸟巢(国家体育场)</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>265</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>北京欢乐谷</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>266</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>路环岛</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>267</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>深圳地铁</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>268</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>尖东</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>269</v>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>苏州古运河</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>270</v>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>香港科学馆</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>271</v>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>南京总统府</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
-        <v>272</v>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>鼓浪屿</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
-        <v>273</v>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>澳门旅游塔会展娱乐中心</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>274</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>沈阳故宫</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>275</v>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>中国国家博物馆</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>276</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>圣保罗大教堂遗址(大三巴牌坊)</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>277</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>平安寨</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>278</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Elysian Tour</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
-        <v>279</v>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>澳门博物馆</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
-        <v>280</v>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>西望洋主教堂</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
-        <v>281</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>丽江木府</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="n">
-        <v>282</v>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>田子坊</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="n">
-        <v>283</v>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>旺角</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="n">
-        <v>284</v>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>西溪湿地公园</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="n">
-        <v>285</v>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>日月塔</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="n">
-        <v>286</v>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>洱海湖</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="n">
-        <v>287</v>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>九龙城寨公园</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="n">
-        <v>288</v>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>翠湖</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="n">
-        <v>289</v>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>洪崖洞</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="n">
-        <v>290</v>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>拙政园</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="n">
-        <v>291</v>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>黄大仙祠</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="n">
-        <v>292</v>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>天津之眼摩天轮</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="n">
-        <v>293</v>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>三亚珠江南田温泉</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="n">
-        <v>294</v>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>大明湖公园</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="n">
-        <v>295</v>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>三峡博物馆</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="n">
-        <v>296</v>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>世纪公园</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="n">
-        <v>297</v>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>前门大街商业街</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="n">
-        <v>298</v>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>芦笛岩</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="n">
-        <v>299</v>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>东望洋炮台</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="n">
-        <v>300</v>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>海港城</t>
+          <t>黄浦江</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh attractionsFromPage Excel and recording from pages 2–6 scrape
Co-authored-by: 吴志中 <wuzhizhong1@xdf.cn>
</commit_message>
<xml_diff>
--- a/attractionsFromPage.xlsx
+++ b/attractionsFromPage.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B150"/>
+  <dimension ref="A1:B151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,1491 +430,1501 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>151</v>
+        <v>31</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>中央大街步行街</t>
+          <t>上窰民俗文物馆</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>152</v>
+        <v>32</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>印象丽江</t>
+          <t>国际眼镜城</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>153</v>
+        <v>33</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>崇圣寺三塔</t>
+          <t>西藏高原旅游的一日游</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>154</v>
+        <v>34</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>文殊院</t>
+          <t>香港旅游发展局</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>155</v>
+        <v>35</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>香港西贡</t>
+          <t>Sandbox - 沙盒 VR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>156</v>
+        <v>36</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>广州地铁</t>
+          <t>南外滩轻纺面料市场</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>157</v>
+        <v>37</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>上海城市历史发展陈列馆</t>
+          <t>布达拉宫</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>158</v>
+        <v>38</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>杭州宋城</t>
+          <t>L&amp;K裁缝</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>159</v>
+        <v>39</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Beijing Airport Layover Tour</t>
+          <t>黄花城长城</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>鹿回头公园</t>
+          <t>张家界国家森林公园</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>161</v>
+        <v>41</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>狮子林</t>
+          <t>Art Alba Gallery</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>162</v>
+        <v>42</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>陈家祠</t>
+          <t>Xianggong Mountain</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>163</v>
+        <v>43</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>网师园</t>
+          <t>云冈石窟</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>164</v>
+        <v>44</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>中国丽江古城</t>
+          <t>南莲园池</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>165</v>
+        <v>45</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>798艺术区</t>
+          <t>九寨沟自然保护区</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>166</v>
+        <v>46</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>香港海事博物馆</t>
+          <t>大熊猫保护研究中心都江堰基地</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>167</v>
+        <v>47</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>东方明珠</t>
+          <t>黑暗中对话</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>168</v>
+        <v>48</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>崂山自然风景区</t>
+          <t>箭扣长城</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>169</v>
+        <v>49</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>汉阳陵</t>
+          <t>黄山</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>170</v>
+        <v>50</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>峨眉山</t>
+          <t>慈山寺</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>171</v>
+        <v>51</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>同里古镇</t>
+          <t>亚特兰蒂斯水世界</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>172</v>
+        <v>52</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>豫园</t>
+          <t>龙脊梯田</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>173</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>大馆</t>
+          <t>张家界天门山</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>174</v>
+        <v>54</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>云南石林地质公园</t>
+          <t>龙门石窟</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>175</v>
+        <v>55</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>天一阁</t>
+          <t>哈尔滨冰雪大世界</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>176</v>
+        <v>56</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>西湖花港观鱼公园</t>
+          <t>泸沽湖</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>177</v>
+        <v>57</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>金茂大厦</t>
+          <t>居庸关长城</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>178</v>
+        <v>58</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>回坊风情街</t>
+          <t>司马台长城</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>179</v>
+        <v>59</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>花城广场</t>
+          <t>张家界武陵源风景名胜区</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>颐和园佛香阁</t>
+          <t>龙脊</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>181</v>
+        <v>61</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>平江路</t>
+          <t>外滩万国建筑博览</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>182</v>
+        <v>62</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>虎丘</t>
+          <t>志莲净苑</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>183</v>
+        <v>63</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>青海湖</t>
+          <t>悬空寺</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>184</v>
+        <v>64</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>香港文化博物馆</t>
+          <t>莫高窟</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>185</v>
+        <v>65</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>太阳岛</t>
+          <t>Mary’s Xian Tours</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>186</v>
+        <v>66</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>鸣沙山</t>
+          <t>拉萨大昭寺</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>187</v>
+        <v>67</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>玉佛禅寺</t>
+          <t>成都地铁</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>188</v>
+        <v>68</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>凤凰古城</t>
+          <t>Real China Travel</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>189</v>
+        <v>69</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>昆明龙门</t>
+          <t>跑马地赛马场</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>190</v>
+        <v>70</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>金沙遗址博物馆</t>
+          <t>遇龙河</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>191</v>
+        <v>71</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>中华恐龙园</t>
+          <t>长隆国际马戏大剧院</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>192</v>
+        <v>72</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>明孝陵</t>
+          <t>上海中心大厦</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>193</v>
+        <v>73</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>郑家大屋</t>
+          <t>u-bestour</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>194</v>
+        <v>74</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>旧城</t>
+          <t>上海犹太难民纪念馆</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>195</v>
+        <v>75</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Happy Dragon Tour</t>
+          <t>北京八达岭长城</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>196</v>
+        <v>76</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>南京城墙(明城墙)</t>
+          <t>雍和宫</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>197</v>
+        <v>77</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>珠海长隆海洋王国</t>
+          <t>张掖丹霞地质文化公园</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>198</v>
+        <v>78</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>新濠天地</t>
+          <t>景山公园</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>周庄水乡</t>
+          <t>香港电车（叮叮车）</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alex's Epic Xian的一日游</t>
+          <t>漓江景区</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>201</v>
+        <v>81</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>澳门历史城区</t>
+          <t>哲蚌寺</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>202</v>
+        <v>82</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>留园</t>
+          <t>西湖</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>203</v>
+        <v>83</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>香港历史博物馆</t>
+          <t>华山</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>204</v>
+        <v>84</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>陕西历史博物馆</t>
+          <t>飞来峰</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>205</v>
+        <v>85</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>苏州博物馆</t>
+          <t>国家大剧院</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>206</v>
+        <v>86</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>八大关</t>
+          <t>磁悬浮列车</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>207</v>
+        <v>87</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>午门</t>
+          <t>湖北省博物馆</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>208</v>
+        <v>88</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>珠穆朗玛峰基地营</t>
+          <t>上海宣传画艺术中心</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>209</v>
+        <v>89</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>两江四湖景区</t>
+          <t>长隆野生动物园</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>211</v>
+        <v>90</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>长洲岛</t>
+          <t>太和殿</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>212</v>
+        <v>91</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>白云山</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>213</v>
+        <v>92</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>峨眉山金顶</t>
+          <t>南山寺</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>214</v>
+        <v>93</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>澳门大熊猫馆</t>
+          <t>香港维多利亚海港</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>215</v>
+        <v>94</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>朱家角古镇</t>
+          <t>北海公园</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>216</v>
+        <v>95</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>扎什伦布寺</t>
+          <t>云台山地质公园</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>217</v>
+        <v>96</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>古北水镇</t>
+          <t>祈年殿</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>218</v>
+        <v>97</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>武汉东湖</t>
+          <t>八角街</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>219</v>
+        <v>98</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>大雁塔</t>
+          <t>深圳莲花山公园</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>220</v>
+        <v>99</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>锦绣中华·民俗村</t>
+          <t>猫之茶房</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>221</v>
+        <v>100</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>大雁塔北广场</t>
+          <t>云南沙溪古镇</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>222</v>
+        <v>101</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>青岛啤酒博物馆</t>
+          <t>大屿山</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>223</v>
+        <v>102</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>西塘古镇</t>
+          <t>浦东新区</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>224</v>
+        <v>103</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>沙面岛</t>
+          <t>天际100香港观景台</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>225</v>
+        <v>104</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>黄龙名胜风景区</t>
+          <t>西安城墙</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>226</v>
+        <v>105</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>尖沙咀海滨长廊</t>
+          <t>滨江大道</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>227</v>
+        <v>106</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>星海广场</t>
+          <t>成都大熊猫繁育研究基地</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>228</v>
+        <v>107</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>故宫九龙壁</t>
+          <t>上海环球金融中心</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>229</v>
+        <v>108</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Guangzhou Private Local Tour Guide-Lorena</t>
+          <t>虎跳峡</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>230</v>
+        <v>109</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>上海人文历史地貌区</t>
+          <t>朝阳剧场</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>231</v>
+        <v>110</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>复兴公园</t>
+          <t>平遥古城</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>232</v>
+        <v>111</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>岳麓山</t>
+          <t>香港公园</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>233</v>
+        <v>112</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>大澳</t>
+          <t>观光缆车</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>234</v>
+        <v>113</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>外滩城市雕塑群</t>
+          <t>万佛寺</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>235</v>
+        <v>114</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>广州图书馆</t>
+          <t>苏州古典园林</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>236</v>
+        <v>115</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>大芬油画村</t>
+          <t>YakPanda</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>237</v>
+        <v>116</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>趵突泉公园</t>
+          <t>龙华寺</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>238</v>
+        <v>117</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>南丫岛</t>
+          <t>上海自然博物馆(静安新馆)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>239</v>
+        <v>118</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>南普陀寺</t>
+          <t>长隆欢乐世界</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>240</v>
+        <v>119</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>金鸡湖</t>
+          <t>宝莲禅寺</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>241</v>
+        <v>120</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>九龙公园</t>
+          <t>狮子亭观景台</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>242</v>
+        <v>121</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Travel Beijing Guide</t>
+          <t>黄浦江</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>243</v>
+        <v>122</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>三清山</t>
+          <t>宏村</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>244</v>
+        <v>123</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SoHo 荷南美食区</t>
+          <t>Beijing Airport Layover Tour</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>245</v>
+        <v>124</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>后海</t>
+          <t>表演湖</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>246</v>
+        <v>125</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>普陀山</t>
+          <t>亚龙湾</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>247</v>
+        <v>126</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COCO PARK</t>
+          <t>颐和园长廊</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>248</v>
+        <v>127</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>西安博物院</t>
+          <t>松赞林寺</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>249</v>
+        <v>128</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>冈仁波齐峰</t>
+          <t>乐山大佛</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>250</v>
+        <v>129</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>赤柱</t>
+          <t>"鸭灵号"帆船</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>251</v>
+        <v>130</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Beijing Impression Tours</t>
+          <t>青城山</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>252</v>
+        <v>131</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>厦门大学</t>
+          <t>天子山</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>253</v>
+        <v>132</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>孔庙和国子监博物馆</t>
+          <t>乌镇</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>254</v>
+        <v>133</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>成都人民公园</t>
+          <t>珠江新城</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>255</v>
+        <v>134</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>束河古镇</t>
+          <t>玉龙雪山</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>256</v>
+        <v>135</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>China Educational Tours</t>
+          <t>黄果树瀑布</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>257</v>
+        <v>136</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>石室圣心大教堂</t>
+          <t>尖沙咀</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>258</v>
+        <v>137</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>杜甫草堂</t>
+          <t>西汉南越王博物馆</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>259</v>
+        <v>138</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>圆明园</t>
+          <t>羊卓雍措湖</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>260</v>
+        <v>139</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>祖庙</t>
+          <t>广州塔</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>261</v>
+        <v>140</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>珠江</t>
+          <t>灵山大佛</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>262</v>
+        <v>141</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>上海虹桥火车站</t>
+          <t>玄武湖</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>263</v>
+        <v>142</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>元阳梯田</t>
+          <t>澳门旅游塔</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>264</v>
+        <v>143</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>鸟巢(国家体育场)</t>
+          <t>上海城市规划展示馆</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>265</v>
+        <v>144</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>北京欢乐谷</t>
+          <t>色拉寺</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>266</v>
+        <v>145</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>路环岛</t>
+          <t>都江堰水利工程</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>267</v>
+        <v>146</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>深圳地铁</t>
+          <t>瘦西湖</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>268</v>
+        <v>147</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>尖东</t>
+          <t>日月双塔文化公园</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>269</v>
+        <v>148</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>苏州古运河</t>
+          <t>中山陵</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>270</v>
+        <v>149</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>香港科学馆</t>
+          <t>故宫御花园</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>271</v>
+        <v>150</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>南京总统府</t>
+          <t>泰山</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>272</v>
+        <v>151</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>鼓浪屿</t>
+          <t>中央大街步行街</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>273</v>
+        <v>152</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>澳门旅游塔会展娱乐中心</t>
+          <t>中国丽江古城</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>274</v>
+        <v>153</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>沈阳故宫</t>
+          <t>上海博物馆</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>275</v>
+        <v>154</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>中国国家博物馆</t>
+          <t>崇圣寺三塔</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>276</v>
+        <v>155</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>圣保罗大教堂遗址(大三巴牌坊)</t>
+          <t>文殊院</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>277</v>
+        <v>156</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>平安寨</t>
+          <t>印象丽江</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>278</v>
+        <v>157</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Elysian Tour</t>
+          <t>陈家祠</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>279</v>
+        <v>158</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>澳门博物馆</t>
+          <t>香港西贡</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>280</v>
+        <v>159</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>西望洋主教堂</t>
+          <t>广州地铁</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>281</v>
+        <v>160</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>丽江木府</t>
+          <t>上海城市历史发展陈列馆</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>282</v>
+        <v>161</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>田子坊</t>
+          <t>狮子林</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>283</v>
+        <v>162</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>旺角</t>
+          <t>网师园</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>284</v>
+        <v>163</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>西溪湿地公园</t>
+          <t>杭州宋城</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>285</v>
+        <v>164</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>日月塔</t>
+          <t>东方明珠</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>286</v>
+        <v>165</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>洱海湖</t>
+          <t>崂山自然风景区</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>287</v>
+        <v>166</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>九龙城寨公园</t>
+          <t>798艺术区</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>288</v>
+        <v>167</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>翠湖</t>
+          <t>鹿回头公园</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>289</v>
+        <v>168</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>洪崖洞</t>
+          <t>香港海事博物馆</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>290</v>
+        <v>169</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>拙政园</t>
+          <t>峨眉山</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>291</v>
+        <v>170</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>黄大仙祠</t>
+          <t>汉阳陵</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>292</v>
+        <v>171</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>天津之眼摩天轮</t>
+          <t>云南石林地质公园</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>293</v>
+        <v>172</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>三亚珠江南田温泉</t>
+          <t>同里古镇</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>294</v>
+        <v>173</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>大明湖公园</t>
+          <t>大馆</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>295</v>
+        <v>174</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>三峡博物馆</t>
+          <t>西湖花港观鱼公园</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>296</v>
+        <v>175</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>世纪公园</t>
+          <t>金茂大厦</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>297</v>
+        <v>176</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>前门大街商业街</t>
+          <t>回坊风情街</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>298</v>
+        <v>177</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>芦笛岩</t>
+          <t>平江路</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>299</v>
+        <v>178</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>东望洋炮台</t>
+          <t>虎丘</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>300</v>
+        <v>179</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>海港城</t>
+          <t>昆明龙门</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>180</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>豫园</t>
         </is>
       </c>
     </row>

</xml_diff>